<commit_message>
fix: add Sprint 4/5 tests (T58-T74) to QA checklist script
make-qa-checklist.js TESTS array was frozen at T01-T57. Entries T58-T74
in qa_status.json were silently ignored and never appeared in the xlsx.
Added two new categories (sprint4, sprint5) with all 17 missing tests.
QA checklist now 74 tests, 73 passing.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NeverMiss_QA_Checklist.xlsx
+++ b/NeverMiss_QA_Checklist.xlsx
@@ -6,7 +6,7 @@
     <sheet name="QA Checklist" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D85</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D66"/>
+  <dimension ref="A1:D85"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="52.83203125" customWidth="1"/>
@@ -1332,10 +1332,276 @@
         <v>src/integrations/payment/payme.ts + ai/claudeClient.ts — stubs מוכנים; BUG-030 תוקן</v>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>🔗</v>
+      </c>
+      <c r="B67" t="str">
+        <v>DeviceContactsScreen — ייבוא מאנשי קשר של המכשיר (Capacitor)</v>
+      </c>
+      <c r="C67" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D67" t="str">
+        <v>BL-030 Sprint 3: DeviceContactsScreen with @capacitor-community/contacts; consent/permission/list/import flow; phone dedup; Capacitor.isNativePlatform() guard; Premium route /device-contacts; import shortcut in ImportContactsScreen</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>🚀</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Sprint 4 — ייצוא / גיבוי / נגישות / ספרינט</v>
+      </c>
+      <c r="C68" t="str">
+        <v/>
+      </c>
+      <c r="D68" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>🚀</v>
+      </c>
+      <c r="B69" t="str">
+        <v>celebrationType שדה בקשר — סינון חגים לפי סוג חגיגה</v>
+      </c>
+      <c r="C69" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D69" t="str">
+        <v>BL-026 Sprint 3: CelebrationType field added to Contact; select in ContactForm Cultural section; CELEBRATION_TO_RELIGION map in scoringSystem.ts; 10 i18n keys EN+HE</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>🚀</v>
+      </c>
+      <c r="B70" t="str">
+        <v>התראה לאיש קשר שלא דיברו עמו 45 יום + יום הולדת קרוב</v>
+      </c>
+      <c r="C70" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D70" t="str">
+        <v>BL-023 Sprint 3: Overdue contact notification added to notificationService.ts (45-day threshold); skips if birthday reminder within 7d; dedup via nm_notif_sent; EN+HE keys</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>🚀</v>
+      </c>
+      <c r="B71" t="str">
+        <v>BUG-043: נקודות חגים מרובי-ימים (סוכות/חנוכה) בלוח שנה</v>
+      </c>
+      <c r="C71" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D71" t="str">
+        <v>BUG-043: CalendarScreen getHolidaysForDay now uses numeric YYYYMMDD range; all days of Sukkot/Hanukkah/multi-day holidays show dot</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>🚀</v>
+      </c>
+      <c r="B72" t="str">
+        <v>BUG-044: סוכות 2026 נוסף ל-holidays.ts</v>
+      </c>
+      <c r="C72" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D72" t="str">
+        <v>BUG-044: sukkot-2026 added to holidays.ts (Sep 25–Oct 2, 2026); calendar now shows Sukkot for 2026</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>🚀</v>
+      </c>
+      <c r="B73" t="str">
+        <v>BL-025: ייצוא אנשי קשר ל-CSV (Premium)</v>
+      </c>
+      <c r="C73" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D73" t="str">
+        <v>BL-025 Sprint 4: exportService.ts עם PapaParse + BOM; כפתור ייצוא CSV ב-SettingsScreen Premium Features; exportDone feedback 2.5s; EN+HE i18n keys</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>🚀</v>
+      </c>
+      <c r="B74" t="str">
+        <v>BL-029: כל כפתורי icon-only ≥ 48×48px (WCAG 2.5.5)</v>
+      </c>
+      <c r="C74" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D74" t="str">
+        <v>BL-029 Sprint 4 WCAG 2.5.5: 9 כפתורי icon-only עודכנו ל-min-w/h-[48px]; Navigation, ContactForm, ContactDetail, GroupsScreen, GreetingEditor, Modal, HolidayDetail, BirthdayGreetingEditor</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>🚀</v>
+      </c>
+      <c r="B75" t="str">
+        <v>BL-024: haptic feedback — שמירת קשר / שליחת ברכה / קופון</v>
+      </c>
+      <c r="C75" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D75" t="str">
+        <v>BL-024 Sprint 4: hapticService.ts עם Light/Medium/Success/Error; מחובר ל-save contact, send greeting (ChannelPicker), coupon success/error; no-op בדפדפן</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>🚀</v>
+      </c>
+      <c r="B76" t="str">
+        <v>BL-034: גיבוי ושחזור JSON (ייצוא/ייבוא כל הנתונים)</v>
+      </c>
+      <c r="C76" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D76" t="str">
+        <v>BL-034 Sprint 4: exportBackupJSON/importBackupJSON ב-storageService.ts; UI ב-SettingsScreen Premium Features; restore reload אוטומטי; error state 3s</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>🚀</v>
+      </c>
+      <c r="B77" t="str">
+        <v>BL-035: זיהוי קשר כפול — שם זהה או מספר טלפון זהה</v>
+      </c>
+      <c r="C77" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D77" t="str">
+        <v>BL-035 Sprint 4: findDuplicate() בודק שם exact + phone ≥7 ספרות; Modal אזהרה עם שם הכפול; Save Anyway / Cancel; לא חוסם עריכה קיימת</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>🗂️</v>
+      </c>
+      <c r="B78" t="str">
+        <v>Sprint 5 — ייבוא / קבוצות / ניווט</v>
+      </c>
+      <c r="C78" t="str">
+        <v/>
+      </c>
+      <c r="D78" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>🗂️</v>
+      </c>
+      <c r="B79" t="str">
+        <v>BL-046: כפתור ייבוא ב-ContactsScreen (Premium) + empty-state shortcut</v>
+      </c>
+      <c r="C79" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D79" t="str">
+        <v>BL-046 Sprint 5: FileUp icon ב-ContactsScreen header (Premium only) + empty-state shortcut → /import</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>🗂️</v>
+      </c>
+      <c r="B80" t="str">
+        <v>BL-047: תוויות CSV בלבד ב-ImportContactsScreen</v>
+      </c>
+      <c r="C80" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D80" t="str">
+        <v>BL-047 Sprint 5: accept='.csv' + תווית 📄 CSV badge + i18n key import_csvOnly ב-ImportContactsScreen</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>🗂️</v>
+      </c>
+      <c r="B81" t="str">
+        <v>BL-048: כפתור import מהמכשיר כ-Blue gradient card</v>
+      </c>
+      <c r="C81" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D81" t="str">
+        <v>BL-048 Sprint 5: כפתור device contacts כ-Blue gradient card עם Smartphone icon + arrow; divider 'or upload CSV' ב-ImportContactsScreen</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>🗂️</v>
+      </c>
+      <c r="B82" t="str">
+        <v>BL-049: מחוון tab פעיל — נקודה / אייקון גדול / טקסט עבה</v>
+      </c>
+      <c r="C82" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D82" t="str">
+        <v>BL-049 Sprint 5: dot indicator + icon 22px + fontWeight 800 primary color label על tab פעיל ב-BottomNav; background glow</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>🗂️</v>
+      </c>
+      <c r="B83" t="str">
+        <v>BL-052: purpose selector בקבוצה + הצעות חגים אוטומטיות</v>
+      </c>
+      <c r="C83" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D83" t="str">
+        <v>BL-052 Sprint 5: GroupPurpose type + purpose field ב-Group; SUGGESTED_BASES lookup; applyPurpose(); purpose pills + ✦ badge על holidays מוצעים ב-GroupsScreen</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>🗂️</v>
+      </c>
+      <c r="B84" t="str">
+        <v>BL-050: שיוך אנשי קשר מיובאים לקבוצה בשלב done</v>
+      </c>
+      <c r="C84" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D84" t="str">
+        <v>BL-050 Sprint 5: group assignment UI בשלב done של ImportContactsScreen; select + assign button; Set merge; groupAssigned success state</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>🗂️</v>
+      </c>
+      <c r="B85" t="str">
+        <v>BL-051: הורדת תבנית CSV עם כותרות עבריות</v>
+      </c>
+      <c r="C85" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D85" t="str">
+        <v>BL-051 Sprint 5: downloadCSVTemplate() — CSV Blob עם BOM + עמודות עבריות + שורת דוגמה; כפתור בשלב upload</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D66"/>
+  <autoFilter ref="A1:D85"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D66"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D85"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sprint 6: quality fixes — FINDING 31/49/75/76/84/85/86
- FINDING 86: Extract SUGGESTED_BASES to src/data/groupSuggestions.ts
- FINDING 75/87: applyPurpose() prunes previous-purpose holiday suggestions
- FINDING 31: Remove redundant hardcoded "1:00" from recording UI (media_record_limit key is self-describing)
- FINDING 49: "Send to group" CTA navigates to /greeting?contactId=&holidayId= instead of generic /contacts
- FINDING 76/81: findDuplicate() covers edits with self-exclusion by contact ID; handleSave checks on both new+edit
- FINDING 84/85: Group assign card hidden when 0 contacts imported; assign button has try/catch + Hebrew error toast
- i18n: import_groupAssignError key added (EN+HE)
- QA: 80 tests, 79✅ 1⚠️ 0❌; changelog.xlsx 166 entries

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NeverMiss_QA_Checklist.xlsx
+++ b/NeverMiss_QA_Checklist.xlsx
@@ -6,7 +6,7 @@
     <sheet name="QA Checklist" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D92</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D85"/>
+  <dimension ref="A1:D92"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="52.83203125" customWidth="1"/>
@@ -1598,10 +1598,108 @@
         <v>BL-051 Sprint 5: downloadCSVTemplate() — CSV Blob עם BOM + עמודות עבריות + שורת דוגמה; כפתור בשלב upload</v>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>🔧</v>
+      </c>
+      <c r="B86" t="str">
+        <v>Sprint 6 — תיקוני איכות / Findings 31/49/75/76/84/85/86</v>
+      </c>
+      <c r="C86" t="str">
+        <v/>
+      </c>
+      <c r="D86" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>🔧</v>
+      </c>
+      <c r="B87" t="str">
+        <v>FINDING 86: SUGGESTED_BASES חולץ ל-src/data/groupSuggestions.ts</v>
+      </c>
+      <c r="C87" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D87" t="str">
+        <v>FINDING 86 Sprint 6: SUGGESTED_BASES חולץ ל-src/data/groupSuggestions.ts; GroupsScreen מייבא ממנו</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>🔧</v>
+      </c>
+      <c r="B88" t="str">
+        <v>FINDING 75/87: applyPurpose מנקה holidays של קטגוריה קודמת</v>
+      </c>
+      <c r="C88" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D88" t="str">
+        <v>FINDING 75/87 Sprint 6: applyPurpose() מנקה ה-holidays מהקטגוריה הישנה לפני הוספת החדשים — אין הצטברות של holidays לא רלוונטיים</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>🔧</v>
+      </c>
+      <c r="B89" t="str">
+        <v>FINDING 31: MediaAttachmentPicker — "1:00" מיותר הוסר</v>
+      </c>
+      <c r="C89" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D89" t="str">
+        <v>FINDING 31 Sprint 6: MediaAttachmentPicker — הוסרו המילים " 1:00" המיותרות; ממשק ההקלטה מציג רק t(media_record_limit)</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>🔧</v>
+      </c>
+      <c r="B90" t="str">
+        <v>FINDING 49: Send to Group מנווט ל-/greeting עם contactId+holidayId</v>
+      </c>
+      <c r="C90" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D90" t="str">
+        <v>FINDING 49 Sprint 6: כפתור Send to Group מנווט ל-/greeting עם contactId + holidayId של איש הקשר הראשון בקבוצה</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>🔧</v>
+      </c>
+      <c r="B91" t="str">
+        <v>FINDING 76/81: findDuplicate בודקת עריכה + self-exclusion</v>
+      </c>
+      <c r="C91" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D91" t="str">
+        <v>FINDING 76/81 Sprint 6: findDuplicate() בודקת גם עת עריכה; self-exclusion לפי contact.id; handleSave ללא גייט isNew</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>🔧</v>
+      </c>
+      <c r="B92" t="str">
+        <v>FINDING 84/85: group assign try/catch + hidden when 0 imported</v>
+      </c>
+      <c r="C92" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D92" t="str">
+        <v>FINDING 84/85 Sprint 6: כרטיס שיוך קבוצה מוסתר כשאין קשרים מיובאים; כפתור שיוך עם try/catch + הודעת שגיאה בעברית</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D85"/>
+  <autoFilter ref="A1:D92"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D85"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D92"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sprint 8: RTL/i18n correctness + WCAG accessibility fixes (FINDING 28D, 29A/B/C)
- FINDING 28D: Add dir(langCode) to i18n/index.ts (RTL_LANG_CODES Set); GreetingRow
  gains langCode prop; dir attribute derived from dir(langCode) — no more fragile
  string comparison against translated display labels
- FINDING 29A: contactForm_avatarColor key (EN+HE); replace hardcoded 'Avatar Color'
- FINDING 29B: contactForm_autoGradient key (EN+HE); replace title= with aria-label=
  on icon-only button (WCAG 4.1.2 fix)
- FINDING 29C: confirmed PremiumFeaturePrompt already uses t('premium_feat_birthday_fields')
- BACKLOG: BL-032 rescheduled to Sprint 9; BL-033 rescheduled to Sprint 10
- changelog.xlsx (184→189 entries), QA checklist (88→93 tests, 91 passing)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NeverMiss_QA_Checklist.xlsx
+++ b/NeverMiss_QA_Checklist.xlsx
@@ -6,7 +6,7 @@
     <sheet name="QA Checklist" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D107</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D101"/>
+  <dimension ref="A1:D107"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="52.83203125" customWidth="1"/>
@@ -1822,10 +1822,94 @@
         <v>Sprint 7 QA: בדיקת מצב הדגמה end-to-end — Onboarding → Try Demo → DemoBanner → Settings exit; RTL Hebrew; בידוד נתונים</v>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>🔧</v>
+      </c>
+      <c r="B102" t="str">
+        <v>Sprint 8 — Stability · Accessibility · RTL/Hebrew Correctness (FINDING 28D, 29A/B/C)</v>
+      </c>
+      <c r="C102" t="str">
+        <v/>
+      </c>
+      <c r="D102" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>🔧</v>
+      </c>
+      <c r="B103" t="str">
+        <v>FINDING 28D: dir(langCode) ב-i18n; GreetingRow dir attribute מחושב לפי langCode</v>
+      </c>
+      <c r="C103" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D103" t="str">
+        <v>Sprint 8 FINDING 28D: dir(langCode) נוסף ל-src/i18n/index.ts; GreetingRow משתמשת ב-langCode prop במקום השוואת מחרוזת; build+lint עבר</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>🔧</v>
+      </c>
+      <c r="B104" t="str">
+        <v>FINDING 29A: תווית Avatar Color מוחלפת ב-t(contactForm_avatarColor) — EN/HE</v>
+      </c>
+      <c r="C104" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D104" t="str">
+        <v>Sprint 8 FINDING 29A: תווית 'Avatar Color' מוחלפת ב-t('contactForm_avatarColor') — EN/HE תוקן</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>🔧</v>
+      </c>
+      <c r="B105" t="str">
+        <v>FINDING 29B: aria-label על כפתור Auto gradient — WCAG 4.1.2 תוקן</v>
+      </c>
+      <c r="C105" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D105" t="str">
+        <v>Sprint 8 FINDING 29B: כפתור 'Auto gradient' — title הוחלף ב-aria-label={t('contactForm_autoGradient')}; WCAG 4.1.2 מתוקן</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>🔧</v>
+      </c>
+      <c r="B106" t="str">
+        <v>FINDING 29C: PremiumFeaturePrompt feature — t(premium_feat_birthday_fields) כבר קיים</v>
+      </c>
+      <c r="C106" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D106" t="str">
+        <v>Sprint 8 FINDING 29C: PremiumFeaturePrompt feature כבר שימשה ב-t('premium_feat_birthday_fields') — לא נדרש שינוי</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>🔧</v>
+      </c>
+      <c r="B107" t="str">
+        <v>Sprint 8 QA: build נקי + lint נקי אחרי כל תיקוני Sprint 8</v>
+      </c>
+      <c r="C107" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D107" t="str">
+        <v>Sprint 8 QA: build עבר ו-lint נקי אחרי כל תיקוני Sprint 8</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D101"/>
+  <autoFilter ref="A1:D107"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D101"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D107"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sprint 11: Quick Send panel (BL-064) + tone auto-regenerate + Hebrew template fixes (BL-063)
BL-063 — Fix greeting generation logic:
- GreetingEditorScreen: useEffect([tone]) triggers generate() on tier change (BUG-047)
- greetingService.ts: fix Hebrew friendly generic templates — 'לברר'→'לדעת', 'שכל טוב'→'שיהיה הכל טוב' (BUG-048)

BL-064 — One-tap Quick Send from Dashboard:
- DashboardScreen: Quick Send overlay (fixed-bottom panel) with 3 AI-generated options per contact
- Birthday cards + group holiday alerts show 'שלח ברכה' CTA button
- Per-option: WhatsApp, Copy, Open Editor actions; premium gate
- i18n: 8 dashboard_quick_send_* keys EN+HE

QA: 113 tests — 111 ✅ | 1 ⚠️ | 1 ☐

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NeverMiss_QA_Checklist.xlsx
+++ b/NeverMiss_QA_Checklist.xlsx
@@ -6,7 +6,7 @@
     <sheet name="QA Checklist" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D122</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D130</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D122"/>
+  <dimension ref="A1:D130"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="52.83203125" customWidth="1"/>
@@ -2116,10 +2116,122 @@
         <v>BL-060: כל התאריכים החדשים עם religion: Secular; ברכות EN+HE; הערות רגישות לתאריכי אבל; build+lint נקי</v>
       </c>
     </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>✉️</v>
+      </c>
+      <c r="B123" t="str">
+        <v>Sprint 11 — Quick Send (BL-064) + Auto-Regenerate on Tone (BL-063) + UpgradeScreen CTA Fix (BL-062)</v>
+      </c>
+      <c r="C123" t="str">
+        <v/>
+      </c>
+      <c r="D123" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>✉️</v>
+      </c>
+      <c r="B124" t="str">
+        <v>BL-063 / BUG-047: useEffect([tone]) — שינוי tier מחולל generate() מחדש אוטומטית ב-GreetingEditorScreen</v>
+      </c>
+      <c r="C124" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D124" t="str">
+        <v>BL-063 / BUG-047: useEffect([tone]) נוסף ל-GreetingEditorScreen — שינוי tier מפעיל generate() מחדש אוטומטית</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>✉️</v>
+      </c>
+      <c r="B125" t="str">
+        <v>BL-063 / BUG-048: תבניות עברית friendly תוקנו — "לברר"→"לדעת", "שכל טוב"→"שיהיה הכל טוב"</v>
+      </c>
+      <c r="C125" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D125" t="str">
+        <v>BL-063 / BUG-048: תבניות עברית friendly תוקנו — 'לברר'→'לדעת', 'שכל טוב'→'שיהיה הכל טוב'; business 'שלחתי ידו/ת'→'פניתי'</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>✉️</v>
+      </c>
+      <c r="B126" t="str">
+        <v>BL-062 / BUG-045: UpgradeScreen CTA — t("upgrade_cta") במקום t("payme_goPayMe"); גנרי ולא תלוי ספק</v>
+      </c>
+      <c r="C126" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D126" t="str">
+        <v>BL-062 / BUG-045: UpgradeScreen CTA עכשיו משתמש ב-t('upgrade_cta') — 'שדרג עכשיו' — לא תלוי ב-PayMe</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>✉️</v>
+      </c>
+      <c r="B127" t="str">
+        <v>BL-062 / BUG-046: upgrade_unlockEverything HE = "שדרג לפרמיום"; upgrade_cta EN/HE נוסף ל-i18n</v>
+      </c>
+      <c r="C127" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D127" t="str">
+        <v>BL-062 / BUG-046: upgrade_unlockEverything HE שונה ל-'שדרג לפרמיום'; upgrade_cta EN/HE נוסף ל-i18n</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>✉️</v>
+      </c>
+      <c r="B128" t="str">
+        <v>BL-064: כפתור "שלח ברכה" על כרטיסי ימי הולדת + קבוצה; premium → Quick Send; free → /greeting</v>
+      </c>
+      <c r="C128" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D128" t="str">
+        <v>BL-064: כפתור 'שלח ברכה' על כרטיסי ימי הולדת + כרטיסי קבוצה; premium → openQuickSend; free → navigate to /greeting</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>✉️</v>
+      </c>
+      <c r="B129" t="str">
+        <v>BL-064: Quick Send overlay — 3 options AI; WhatsApp/Copy/Open Editor לכל option; backdrop סגירה; copied feedback 2s</v>
+      </c>
+      <c r="C129" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D129" t="str">
+        <v>BL-064: Quick Send overlay — 3 options AI per contact; WhatsApp/Copy/Open Editor לכל option; backdrop סגירה; copiedIdx feedback 2s</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>✉️</v>
+      </c>
+      <c r="B130" t="str">
+        <v>Sprint 11 QA: build נקי + lint נקי; BL-062, BL-063, BL-064 מאומתים</v>
+      </c>
+      <c r="C130" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D130" t="str">
+        <v>Sprint 11 QA: build נקי + lint נקי; BL-062+063+064 מיושמים ומאומתים</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D122"/>
+  <autoFilter ref="A1:D130"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D122"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D130"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(BUG-050): add Upgrade Now CTA above coupon section in UpgradeScreen
- Added full-width h-14 gradient button using t('upgrade_now') immediately above
  the coupon section in UpgradeScreen.tsx
- Added upgrade_now i18n key in both EN ('Upgrade Now') and HE ('שדרג עכשיו')
- Button navigates to /payment; coupon section and continue-free untouched
- Updated BUG_REPORT.md (BUG-050), changelog_queue.json, changelog.xlsx, QA checklist

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NeverMiss_QA_Checklist.xlsx
+++ b/NeverMiss_QA_Checklist.xlsx
@@ -6,7 +6,7 @@
     <sheet name="QA Checklist" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D138</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D142</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D138"/>
+  <dimension ref="A1:D142"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="52.83203125" customWidth="1"/>
@@ -2340,10 +2340,66 @@
         <v>Sprint 12 QA: build נקי + lint נקי; BL-067 + BL-065 מיושמים ומאומתים</v>
       </c>
     </row>
+    <row r="139">
+      <c r="A139" t="str">
+        <v>🐞</v>
+      </c>
+      <c r="B139" t="str">
+        <v>Bug Fixes &amp; Improvements — Sprint Suspension Mode</v>
+      </c>
+      <c r="C139" t="str">
+        <v/>
+      </c>
+      <c r="D139" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="str">
+        <v>🐞</v>
+      </c>
+      <c r="B140" t="str">
+        <v>RTL לוח שנה: חצים מוחלפים בעברית (prev=ימין, next=שמאל); LTR ללא שינוי</v>
+      </c>
+      <c r="C140" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D140" t="str">
+        <v>RTL calendar arrows: ChevronLeft/Right מוחלפים כשlang==='he'; prev button מימין, next משמאל בעברית; LTR — ללא שינוי</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="str">
+        <v>🐞</v>
+      </c>
+      <c r="B141" t="str">
+        <v>יום הולדת עברי: dropdown גמטריה; תצוגה כ״א בטבת; Hebrew+Gregorian — 2 אירועים עצמאיים</v>
+      </c>
+      <c r="C141" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D141" t="str">
+        <v>Hebrew birthday: day dropdown מציג גמטריה (א–ל); תצוגה בפורמט כ״א בטבת ב-ContactDetailScreen; Hebrew+Gregorian מטופלים כ-2 אירועים עצמאיים בלוח השנה</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="str">
+        <v>🐞</v>
+      </c>
+      <c r="B142" t="str">
+        <v>BUG-049: PaymeScreen demo mode — באנר הדגמה + כפתור הפעל פרימיום; לא נדרש תשלום אמיתי</v>
+      </c>
+      <c r="C142" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D142" t="str">
+        <v>BUG-049: PaymeScreen שוכתב כ-demo mode; באנר 'זוהי גרסת הדגמה'; כפתור 'הפעל פרימיום (הדגמה)' → activatePremium() + navigate('/dashboard'); build+lint ✅</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D138"/>
+  <autoFilter ref="A1:D142"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D138"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D142"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Bug Fix: Google Translate override, Hebrew holiday descriptions, group form holiday list
BUG-059: Block Google Translate from overriding app language — translate=no + notranslate on html/root
BUG-060: Holiday descriptions always English — added heDescription to all 46 holidays; HolidayDetailScreen shows Hebrew when active
BUG-061: Group form holiday list had duplicates + English-only names/religion — deduplicated by base ID, localized names and religion labels
BUG-057: Hebrew birthday dropdowns already fixed in prior commit (confirmed, no change needed)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NeverMiss_QA_Checklist.xlsx
+++ b/NeverMiss_QA_Checklist.xlsx
@@ -6,7 +6,7 @@
     <sheet name="QA Checklist" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D142</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D145</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D142"/>
+  <dimension ref="A1:D145"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="52.83203125" customWidth="1"/>
@@ -2396,10 +2396,52 @@
         <v>BUG-049: PaymeScreen שוכתב כ-demo mode; באנר 'זוהי גרסת הדגמה'; כפתור 'הפעל פרימיום (הדגמה)' → activatePremium() + navigate('/dashboard'); build+lint ✅</v>
       </c>
     </row>
+    <row r="143">
+      <c r="A143" t="str">
+        <v>🐞</v>
+      </c>
+      <c r="B143" t="str">
+        <v>BUG-059: Google Translate — translate=no + notranslate על html ו-root מונעים תרגום אוטומטי</v>
+      </c>
+      <c r="C143" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D143" t="str">
+        <v>BUG-059 תוקן — translate=no + notranslate על html/root מונעים Google Translate</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="str">
+        <v>🐞</v>
+      </c>
+      <c r="B144" t="str">
+        <v>BUG-060: תיאורי חגים בעברית — heDescription ב-46 חגים; HolidayDetailScreen מציג עברית כשheLang</v>
+      </c>
+      <c r="C144" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D144" t="str">
+        <v>BUG-060 תוקן — heDescription הוסף לכל 46 חגים; HolidayDetailScreen מציג עברית כששפה=he</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="str">
+        <v>🐞</v>
+      </c>
+      <c r="B145" t="str">
+        <v>BUG-061: קבוצות — רשימת חגים ללא כפילויות; שמות עבריים; דת מתורגמת</v>
+      </c>
+      <c r="C145" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D145" t="str">
+        <v>BUG-061 תוקן — GroupsScreen מציג חג ייחודי אחד (ללא כפילות שנה), שם עברי כשhe, דת מתורגמת</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D142"/>
+  <autoFilter ref="A1:D145"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D142"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D145"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: enforce bug lifecycle rule — add BUG-keyed entries to qa_status.json
Per new bug lifecycle rule: each fixed bug now gets a BUG-XXX entry in
qa_status.json with status:fixed + fixedAt timestamp, plus a corresponding
T-entry for the QA checklist. Added BUG-074/075/076 + T127/T128/T129.
QA checklist now shows 129 tests (127 passing).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NeverMiss_QA_Checklist.xlsx
+++ b/NeverMiss_QA_Checklist.xlsx
@@ -6,7 +6,7 @@
     <sheet name="QA Checklist" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D145</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D148</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D145"/>
+  <dimension ref="A1:D148"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="52.83203125" customWidth="1"/>
@@ -2438,10 +2438,52 @@
         <v>BUG-061 תוקן — GroupsScreen מציג חג ייחודי אחד (ללא כפילות שנה), שם עברי כשhe, דת מתורגמת</v>
       </c>
     </row>
+    <row r="146">
+      <c r="A146" t="str">
+        <v>🐞</v>
+      </c>
+      <c r="B146" t="str">
+        <v>BUG-074: Input — מיקום אייקון RTL-aware (ימין בעברית, שמאל באנגלית); ריפוד מותאם</v>
+      </c>
+      <c r="C146" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D146" t="str">
+        <v>BUG-074 תוקן — Input.tsx: useLang + isRTL; אייקון ב-right-3/left-3 בהתאם לכיוון; ריפוד pr-10/pl-10 מתאים. build+lint ✅</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="str">
+        <v>🐞</v>
+      </c>
+      <c r="B147" t="str">
+        <v>BUG-075: PrivacyScreen — 10 סעיפים + hero/badge/intro/footer מתורגמים לעברית (25 מפתחות i18n)</v>
+      </c>
+      <c r="C147" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D147" t="str">
+        <v>BUG-075 תוקן — PrivacyScreen: SECTIONS הועבר לתוך הקומפוננטה; 25 מפתחות i18n חדשים (EN+HE) לכל הכותרות, גוף הטקסט, hero, badge, intro, footer. build+lint ✅</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="str">
+        <v>🐞</v>
+      </c>
+      <c r="B148" t="str">
+        <v>BUG-076: מחלקות CSS פיזיות (ml-*/mr-*/text-right) הוחלפו במחלקות לוגיות (ms-*/me-*/text-end) ב-6 קבצים</v>
+      </c>
+      <c r="C148" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D148" t="str">
+        <v>BUG-076 תוקן — מחלקות CSS פיזיות (ml-*/mr-*/text-right) הוחלפו במחלקות לוגיות (ms-*/me-*/text-end) ב-BirthdayGreetingEditorScreen, App.tsx, DashboardScreen, MediaAttachmentPicker, GreetingEditorScreen, WhatsNewScreen, CalendarScreen. build+lint ✅</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D145"/>
+  <autoFilter ref="A1:D148"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D145"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D148"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(BUG-078): Voice message UX — show manual-attach popup after WhatsApp opens
WhatsApp cannot attach audio via URL. When a voice recording exists and
the user opens WhatsApp, a Modal now appears explaining they must save
and attach the file manually. Modal stays visible until dismissed and is
RTL-ready. Added to both ChannelPicker and WhatsAppButton.

BUG-077 (emoji encoding) verified: encodeURIComponent already present
in buildWhatsAppUrl at all WhatsApp call sites. No code change needed.

New i18n keys: whatsapp_voice_hint_title, whatsapp_voice_hint_body (EN+HE)
Backlog: BL-071 (verified), BL-072 (fixed)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NeverMiss_QA_Checklist.xlsx
+++ b/NeverMiss_QA_Checklist.xlsx
@@ -6,7 +6,7 @@
     <sheet name="QA Checklist" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D148</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D150</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D148"/>
+  <dimension ref="A1:D150"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="52.83203125" customWidth="1"/>
@@ -2480,10 +2480,38 @@
         <v>BUG-076 תוקן — מחלקות CSS פיזיות (ml-*/mr-*/text-right) הוחלפו במחלקות לוגיות (ms-*/me-*/text-end) ב-BirthdayGreetingEditorScreen, App.tsx, DashboardScreen, MediaAttachmentPicker, GreetingEditorScreen, WhatsNewScreen, CalendarScreen. build+lint ✅</v>
       </c>
     </row>
+    <row r="149">
+      <c r="A149" t="str">
+        <v>🐞</v>
+      </c>
+      <c r="B149" t="str">
+        <v>BUG-077: WhatsApp emoji encoding — אומת: encodeURIComponent קיים ב-buildWhatsAppUrl; כל נתיבי השליחה מוסדרים דרכו</v>
+      </c>
+      <c r="C149" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D149" t="str">
+        <v>BUG-077 אומת — buildWhatsAppUrl משתמש ב-encodeURIComponent; כל נתיבי WhatsApp (ChannelPicker, WhatsAppButton, DashboardScreen) עוברים דרך openWhatsApp → buildWhatsAppUrl. אין שינוי קוד נדרש.</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="str">
+        <v>🐞</v>
+      </c>
+      <c r="B150" t="str">
+        <v>BUG-078: Voice message — Modal "צירוף ידני" מוצג לאחר פתיחת WhatsApp כשיש הקלטה; RTL; נשאר עד סגירה ידנית</v>
+      </c>
+      <c r="C150" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D150" t="str">
+        <v>BUG-078 תוקן — Modal הקלטה קולית נוסף ל-ChannelPicker ו-WhatsAppButton; מופיע לאחר פתיחת WhatsApp כשmedia.type===audio; נשאר עד סגירה ידנית; RTL; 2 מפתחות i18n (EN+HE). build+lint ✅</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D148"/>
+  <autoFilter ref="A1:D150"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D148"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D150"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(BL-073/BL-074): add missing Jewish holidays and deduplicate Event Type dropdown
BUG-079 (BL-074): Added 14 missing Jewish holiday entries to holidays.ts —
Lag Ba'Omer, Simchat Torah, Tisha B'Av, 17th of Tammuz, 10th of Tevet,
Fast of Esther, Fast of Gedaliah — 2025+2026 pairs each. Uses hebcalDate()
for accurate Hebrew-calendar dates. Types: fast/minor/major with EN+HE.

BUG-080 (BL-073): Fixed duplicate holiday names in GreetingEditorScreen
Event Type dropdown — added useMemo dedup by name (upcoming-first).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NeverMiss_QA_Checklist.xlsx
+++ b/NeverMiss_QA_Checklist.xlsx
@@ -6,7 +6,7 @@
     <sheet name="QA Checklist" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D150</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D152</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D150"/>
+  <dimension ref="A1:D152"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="52.83203125" customWidth="1"/>
@@ -2508,10 +2508,38 @@
         <v>BUG-078 תוקן — Modal הקלטה קולית נוסף ל-ChannelPicker ו-WhatsAppButton; מופיע לאחר פתיחת WhatsApp כשmedia.type===audio; נשאר עד סגירה ידנית; RTL; 2 מפתחות i18n (EN+HE). build+lint ✅</v>
       </c>
     </row>
+    <row r="151">
+      <c r="A151" t="str">
+        <v>🐞</v>
+      </c>
+      <c r="B151" t="str">
+        <v>BUG-079: 14 חגים יהודיים חסרים נוספו — ל"ג בעומר, שמחת תורה, תשעה באב, י"ז בתמוז, י' בטבת, תענית אסתר, צום גדליה (2025+2026); hebcalDate(); type fast/minor/major</v>
+      </c>
+      <c r="C151" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D151" t="str">
+        <v>BUG-079 תוקן — 14 רשומות חגים יהודיים חסרים נוספו ל-holidays.ts: ל"ג בעומר, שמחת תורה, תשעה באב, י"ז בתמוז, י' בטבת, תענית אסתר, צום גדליה — 2 שנים לכל חג; hebcalDate() לתאריכים מדויקים; type: fast/minor/major; EN+HE. build+lint ✅</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="str">
+        <v>🐞</v>
+      </c>
+      <c r="B152" t="str">
+        <v>BUG-080: כפילויות חגים ב-Event Type dropdown — useMemo dedup by name (upcoming-first) ב-GreetingEditorScreen</v>
+      </c>
+      <c r="C152" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D152" t="str">
+        <v>BUG-080 תוקן — GreetingEditorScreen: useMemo dedup holidays by name (upcoming-first) — כל חג מופיע פעם אחת בתפריט Event Type. build+lint ✅</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D150"/>
+  <autoFilter ref="A1:D152"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D150"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D152"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(BL-077): replace static Jewish holiday dates with dynamic Hebcal generation
17 HebrewTemplates cover all major holidays, fasts, and Israeli national days.
@hebcal/core Israel mode resolves each date at runtime for YEAR_RANGE = [year-1..year+2].
Static Gregorian holidays (Christmas, Islam, etc.) remain unchanged.
Holiday IDs, interface contract, and all exports are backward-compatible.
build + lint clean; 135 QA tests (133 ✅).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NeverMiss_QA_Checklist.xlsx
+++ b/NeverMiss_QA_Checklist.xlsx
@@ -6,7 +6,7 @@
     <sheet name="QA Checklist" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D152</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D154</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D152"/>
+  <dimension ref="A1:D154"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="52.83203125" customWidth="1"/>
@@ -2536,10 +2536,38 @@
         <v>BUG-080 תוקן — GreetingEditorScreen: useMemo dedup holidays by name (upcoming-first) — כל חג מופיע פעם אחת בתפריט Event Type. build+lint ✅</v>
       </c>
     </row>
+    <row r="153">
+      <c r="A153" t="str">
+        <v>⚡</v>
+      </c>
+      <c r="B153" t="str">
+        <v>Sprint 14 — חגים דינמיים BL-077 (Hebcal)</v>
+      </c>
+      <c r="C153" t="str">
+        <v/>
+      </c>
+      <c r="D153" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="str">
+        <v>⚡</v>
+      </c>
+      <c r="B154" t="str">
+        <v>BL-077: חגים יהודיים דינמיים — 17 תבניות Hebcal; YEAR_RANGE=[שנה-1..שנה+2]; IDs ו-Holiday interface זהים; build+lint ✅</v>
+      </c>
+      <c r="C154" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D154" t="str">
+        <v>BL-077 הושלם — חגים יהודיים נוצרים דינמית ע״י @hebcal/core; 17 תבניות; YEAR_RANGE=[שנה-1..שנה+2]; IDs ו-Holiday interface זהים; build+lint ✅</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D152"/>
+  <autoFilter ref="A1:D154"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D152"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D154"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(sprint15): BL-046/047/048 — import contacts UX improvements
BL-046: Remove isPremium guard from ContactsScreen import buttons so all users see the import CTA; premium gate remains at route level (/import → UpgradeScreen for free users).
BL-047: Confirmed import_csvOnly label ("כרגע ניתן לייבא קובץ CSV בלבד") already displayed in upload zone; Hebrew i18n verified.
BL-048: Confirmed device contacts blue gradient card already prominent at top of ImportContactsScreen; no code change needed.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NeverMiss_QA_Checklist.xlsx
+++ b/NeverMiss_QA_Checklist.xlsx
@@ -6,7 +6,7 @@
     <sheet name="QA Checklist" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D154</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D158</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D154"/>
+  <dimension ref="A1:D158"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="52.83203125" customWidth="1"/>
@@ -2564,10 +2564,66 @@
         <v>BL-077 הושלם — חגים יהודיים נוצרים דינמית ע״י @hebcal/core; 17 תבניות; YEAR_RANGE=[שנה-1..שנה+2]; IDs ו-Holiday interface זהים; build+lint ✅</v>
       </c>
     </row>
+    <row r="155">
+      <c r="A155" t="str">
+        <v>📥</v>
+      </c>
+      <c r="B155" t="str">
+        <v>Sprint 15 — ייבוא אנשי קשר UX: BL-046, BL-047, BL-048</v>
+      </c>
+      <c r="C155" t="str">
+        <v/>
+      </c>
+      <c r="D155" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="str">
+        <v>📥</v>
+      </c>
+      <c r="B156" t="str">
+        <v>BL-046: כפתור ייבוא אנשי קשר מוצג בכרטיסיית אנשי קשר לכל המשתמשים; גייט Premium נשמר בנתיב /import</v>
+      </c>
+      <c r="C156" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D156" t="str">
+        <v>BL-046 תוקן — כפתור ייבוא בכרטיסיית אנשי קשר מוצג לכל המשתמשים; גייט Premium נשמר בנתיב</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="str">
+        <v>📥</v>
+      </c>
+      <c r="B157" t="str">
+        <v>BL-047: תווית "כרגע ניתן לייבא קובץ CSV בלבד" מוצגת ליד אזור ההעלאה ב-ImportContactsScreen; תרגום עברי קיים</v>
+      </c>
+      <c r="C157" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D157" t="str">
+        <v>BL-047 אומת — תווית CSV בלבד מוצגת ליד אזור ההעלאה; תרגום עברי קיים</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="str">
+        <v>📥</v>
+      </c>
+      <c r="B158" t="str">
+        <v>BL-048: כרטיסיית ייבוא ממכשיר (גרדיאנט כחול, סמארטפון) מוצגת בראש ImportContactsScreen; נגישות ויזואלית מלאה</v>
+      </c>
+      <c r="C158" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D158" t="str">
+        <v>BL-048 אומת — כרטיסיית ייבוא ממכשיר מוצגת בראש המסך עם גרדיאנט כחול ואייקון סמארטפון</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D154"/>
+  <autoFilter ref="A1:D158"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D154"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D158"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(sprint16): BL-067 — personal user layer verified and closed
Full DoD validation: UserSetupScreen (first-launch name prompt), nm_user_name
localStorage persist, personalised dashboard hero (dashboard_hello), pending
greetings context panel with clickable items, graceful empty states.
All i18n keys present EN+HE. Build+lint clean. No code changes needed.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NeverMiss_QA_Checklist.xlsx
+++ b/NeverMiss_QA_Checklist.xlsx
@@ -6,7 +6,7 @@
     <sheet name="QA Checklist" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D158</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D160</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D158"/>
+  <dimension ref="A1:D160"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="52.83203125" customWidth="1"/>
@@ -2620,10 +2620,38 @@
         <v>BL-048 אומת — כרטיסיית ייבוא ממכשיר מוצגת בראש המסך עם גרדיאנט כחול ואייקון סמארטפון</v>
       </c>
     </row>
+    <row r="159">
+      <c r="A159" t="str">
+        <v>👤</v>
+      </c>
+      <c r="B159" t="str">
+        <v>Sprint 16 — שכבת משתמש אישית BL-067: UserSetupScreen, dashboard_hello, pendingItems</v>
+      </c>
+      <c r="C159" t="str">
+        <v/>
+      </c>
+      <c r="D159" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="str">
+        <v>👤</v>
+      </c>
+      <c r="B160" t="str">
+        <v>BL-067: UserSetupScreen first-launch, nm_user_name persist, dashboard_hello/pending/first_greeting EN+HE, pendingItems clickable, empty states graceful; DoD מלא ✅</v>
+      </c>
+      <c r="C160" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D160" t="str">
+        <v>BL-067 DoD מלא אומת — UserSetupScreen first-launch, nm_user_name persist, dashboard_hello/pending/first_greeting keys EN+HE, pendingItems clickable, empty states graceful</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D158"/>
+  <autoFilter ref="A1:D160"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D158"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D160"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(BUG-081): hide Premium labels when TEMP_PREMIUM_UNLOCK is active
Add showPremiumUI = !TEMP_PREMIUM_UNLOCK to AppContext. When false:
- ContactFormScreen: hides Crown icon, amber border, and "פרטי פרמיום" header (fields remain visible)
- SettingsScreen: hides entire "Premium" section (gold banner, Crown icons, "Premium Active"); hides "Premium Features" nav title; replaces Crown with Sparkles on Birthday Center row

Reverting TEMP_PREMIUM_UNLOCK to false fully restores premium UI.
No premium logic, gating, or monetization behavior was modified.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NeverMiss_QA_Checklist.xlsx
+++ b/NeverMiss_QA_Checklist.xlsx
@@ -6,7 +6,7 @@
     <sheet name="QA Checklist" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D160</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D161</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D160"/>
+  <dimension ref="A1:D161"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="52.83203125" customWidth="1"/>
@@ -2538,16 +2538,16 @@
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>⚡</v>
+        <v>🐞</v>
       </c>
       <c r="B153" t="str">
-        <v>Sprint 14 — חגים דינמיים BL-077 (Hebcal)</v>
+        <v>BUG-081: showPremiumUI=!TEMP_PREMIUM_UNLOCK — Crown + "פרמיום" מוסתרים ב-ContactForm ו-Settings כשגייט MVP פתוח; הפיכה ל-false משחזרת הכל</v>
       </c>
       <c r="C153" t="str">
-        <v/>
+        <v>✅</v>
       </c>
       <c r="D153" t="str">
-        <v/>
+        <v>BUG-081 תוקן — showPremiumUI=!TEMP_PREMIUM_UNLOCK; Crown+פרמיום מוסתרים ב-ContactForm ו-Settings; build+lint ✅</v>
       </c>
     </row>
     <row r="154">
@@ -2555,27 +2555,27 @@
         <v>⚡</v>
       </c>
       <c r="B154" t="str">
-        <v>BL-077: חגים יהודיים דינמיים — 17 תבניות Hebcal; YEAR_RANGE=[שנה-1..שנה+2]; IDs ו-Holiday interface זהים; build+lint ✅</v>
+        <v>Sprint 14 — חגים דינמיים BL-077 (Hebcal)</v>
       </c>
       <c r="C154" t="str">
-        <v>✅</v>
+        <v/>
       </c>
       <c r="D154" t="str">
-        <v>BL-077 הושלם — חגים יהודיים נוצרים דינמית ע״י @hebcal/core; 17 תבניות; YEAR_RANGE=[שנה-1..שנה+2]; IDs ו-Holiday interface זהים; build+lint ✅</v>
+        <v/>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v>📥</v>
+        <v>⚡</v>
       </c>
       <c r="B155" t="str">
-        <v>Sprint 15 — ייבוא אנשי קשר UX: BL-046, BL-047, BL-048</v>
+        <v>BL-077: חגים יהודיים דינמיים — 17 תבניות Hebcal; YEAR_RANGE=[שנה-1..שנה+2]; IDs ו-Holiday interface זהים; build+lint ✅</v>
       </c>
       <c r="C155" t="str">
-        <v/>
+        <v>✅</v>
       </c>
       <c r="D155" t="str">
-        <v/>
+        <v>BL-077 הושלם — חגים יהודיים נוצרים דינמית ע״י @hebcal/core; 17 תבניות; YEAR_RANGE=[שנה-1..שנה+2]; IDs ו-Holiday interface זהים; build+lint ✅</v>
       </c>
     </row>
     <row r="156">
@@ -2583,13 +2583,13 @@
         <v>📥</v>
       </c>
       <c r="B156" t="str">
-        <v>BL-046: כפתור ייבוא אנשי קשר מוצג בכרטיסיית אנשי קשר לכל המשתמשים; גייט Premium נשמר בנתיב /import</v>
+        <v>Sprint 15 — ייבוא אנשי קשר UX: BL-046, BL-047, BL-048</v>
       </c>
       <c r="C156" t="str">
-        <v>✅</v>
+        <v/>
       </c>
       <c r="D156" t="str">
-        <v>BL-046 תוקן — כפתור ייבוא בכרטיסיית אנשי קשר מוצג לכל המשתמשים; גייט Premium נשמר בנתיב</v>
+        <v/>
       </c>
     </row>
     <row r="157">
@@ -2597,13 +2597,13 @@
         <v>📥</v>
       </c>
       <c r="B157" t="str">
-        <v>BL-047: תווית "כרגע ניתן לייבא קובץ CSV בלבד" מוצגת ליד אזור ההעלאה ב-ImportContactsScreen; תרגום עברי קיים</v>
+        <v>BL-046: כפתור ייבוא אנשי קשר מוצג בכרטיסיית אנשי קשר לכל המשתמשים; גייט Premium נשמר בנתיב /import</v>
       </c>
       <c r="C157" t="str">
         <v>✅</v>
       </c>
       <c r="D157" t="str">
-        <v>BL-047 אומת — תווית CSV בלבד מוצגת ליד אזור ההעלאה; תרגום עברי קיים</v>
+        <v>BL-046 תוקן — כפתור ייבוא בכרטיסיית אנשי קשר מוצג לכל המשתמשים; גייט Premium נשמר בנתיב</v>
       </c>
     </row>
     <row r="158">
@@ -2611,27 +2611,27 @@
         <v>📥</v>
       </c>
       <c r="B158" t="str">
-        <v>BL-048: כרטיסיית ייבוא ממכשיר (גרדיאנט כחול, סמארטפון) מוצגת בראש ImportContactsScreen; נגישות ויזואלית מלאה</v>
+        <v>BL-047: תווית "כרגע ניתן לייבא קובץ CSV בלבד" מוצגת ליד אזור ההעלאה ב-ImportContactsScreen; תרגום עברי קיים</v>
       </c>
       <c r="C158" t="str">
         <v>✅</v>
       </c>
       <c r="D158" t="str">
-        <v>BL-048 אומת — כרטיסיית ייבוא ממכשיר מוצגת בראש המסך עם גרדיאנט כחול ואייקון סמארטפון</v>
+        <v>BL-047 אומת — תווית CSV בלבד מוצגת ליד אזור ההעלאה; תרגום עברי קיים</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>👤</v>
+        <v>📥</v>
       </c>
       <c r="B159" t="str">
-        <v>Sprint 16 — שכבת משתמש אישית BL-067: UserSetupScreen, dashboard_hello, pendingItems</v>
+        <v>BL-048: כרטיסיית ייבוא ממכשיר (גרדיאנט כחול, סמארטפון) מוצגת בראש ImportContactsScreen; נגישות ויזואלית מלאה</v>
       </c>
       <c r="C159" t="str">
-        <v/>
+        <v>✅</v>
       </c>
       <c r="D159" t="str">
-        <v/>
+        <v>BL-048 אומת — כרטיסיית ייבוא ממכשיר מוצגת בראש המסך עם גרדיאנט כחול ואייקון סמארטפון</v>
       </c>
     </row>
     <row r="160">
@@ -2639,19 +2639,33 @@
         <v>👤</v>
       </c>
       <c r="B160" t="str">
+        <v>Sprint 16 — שכבת משתמש אישית BL-067: UserSetupScreen, dashboard_hello, pendingItems</v>
+      </c>
+      <c r="C160" t="str">
+        <v/>
+      </c>
+      <c r="D160" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="str">
+        <v>👤</v>
+      </c>
+      <c r="B161" t="str">
         <v>BL-067: UserSetupScreen first-launch, nm_user_name persist, dashboard_hello/pending/first_greeting EN+HE, pendingItems clickable, empty states graceful; DoD מלא ✅</v>
       </c>
-      <c r="C160" t="str">
-        <v>✅</v>
-      </c>
-      <c r="D160" t="str">
+      <c r="C161" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D161" t="str">
         <v>BL-067 DoD מלא אומת — UserSetupScreen first-launch, nm_user_name persist, dashboard_hello/pending/first_greeting keys EN+HE, pendingItems clickable, empty states graceful</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D160"/>
+  <autoFilter ref="A1:D161"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D160"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D161"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(BL-080/BUG-082): correct Israeli holiday notification timing
Replace new Date("YYYY-MM-DD") with parseDateLocal() throughout notificationService.
ISO date strings are parsed as UTC by the browser; in Asia/Jerusalem (UTC+3) this
shifts dates back by 3 hours into the previous day, causing holiday notifications
(Yom HaZikaron, Yom HaAtzmaut) to fire one day early.

parseDateLocal() constructs the date as local midnight (new Date(y, m-1, d)),
eliminating the UTC offset entirely. Also adds explicit safeguards in the holiday
loop: skip if holiday.date is empty or fails to parse. Hebcal Israel mode (il:true)
was already correct — no change needed.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NeverMiss_QA_Checklist.xlsx
+++ b/NeverMiss_QA_Checklist.xlsx
@@ -6,7 +6,7 @@
     <sheet name="QA Checklist" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D161</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D162</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D161"/>
+  <dimension ref="A1:D162"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="52.83203125" customWidth="1"/>
@@ -2552,16 +2552,16 @@
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>⚡</v>
+        <v>🐞</v>
       </c>
       <c r="B154" t="str">
-        <v>Sprint 14 — חגים דינמיים BL-077 (Hebcal)</v>
+        <v>BL-080/BUG-082: parseDateLocal() מחליף new Date(string) — מונע הסטת UTC ב-Asia/Jerusalem; safeguards לתאריך חסר/לא תקין; Hebcal Israel mode אומת כנכון</v>
       </c>
       <c r="C154" t="str">
-        <v/>
+        <v>✅</v>
       </c>
       <c r="D154" t="str">
-        <v/>
+        <v>BL-080 תוקן — parseDateLocal() מונע הסטת UTC; safeguards לתאריך חסר; build+lint ✅</v>
       </c>
     </row>
     <row r="155">
@@ -2569,27 +2569,27 @@
         <v>⚡</v>
       </c>
       <c r="B155" t="str">
-        <v>BL-077: חגים יהודיים דינמיים — 17 תבניות Hebcal; YEAR_RANGE=[שנה-1..שנה+2]; IDs ו-Holiday interface זהים; build+lint ✅</v>
+        <v>Sprint 14 — חגים דינמיים BL-077 (Hebcal)</v>
       </c>
       <c r="C155" t="str">
-        <v>✅</v>
+        <v/>
       </c>
       <c r="D155" t="str">
-        <v>BL-077 הושלם — חגים יהודיים נוצרים דינמית ע״י @hebcal/core; 17 תבניות; YEAR_RANGE=[שנה-1..שנה+2]; IDs ו-Holiday interface זהים; build+lint ✅</v>
+        <v/>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="str">
-        <v>📥</v>
+        <v>⚡</v>
       </c>
       <c r="B156" t="str">
-        <v>Sprint 15 — ייבוא אנשי קשר UX: BL-046, BL-047, BL-048</v>
+        <v>BL-077: חגים יהודיים דינמיים — 17 תבניות Hebcal; YEAR_RANGE=[שנה-1..שנה+2]; IDs ו-Holiday interface זהים; build+lint ✅</v>
       </c>
       <c r="C156" t="str">
-        <v/>
+        <v>✅</v>
       </c>
       <c r="D156" t="str">
-        <v/>
+        <v>BL-077 הושלם — חגים יהודיים נוצרים דינמית ע״י @hebcal/core; 17 תבניות; YEAR_RANGE=[שנה-1..שנה+2]; IDs ו-Holiday interface זהים; build+lint ✅</v>
       </c>
     </row>
     <row r="157">
@@ -2597,13 +2597,13 @@
         <v>📥</v>
       </c>
       <c r="B157" t="str">
-        <v>BL-046: כפתור ייבוא אנשי קשר מוצג בכרטיסיית אנשי קשר לכל המשתמשים; גייט Premium נשמר בנתיב /import</v>
+        <v>Sprint 15 — ייבוא אנשי קשר UX: BL-046, BL-047, BL-048</v>
       </c>
       <c r="C157" t="str">
-        <v>✅</v>
+        <v/>
       </c>
       <c r="D157" t="str">
-        <v>BL-046 תוקן — כפתור ייבוא בכרטיסיית אנשי קשר מוצג לכל המשתמשים; גייט Premium נשמר בנתיב</v>
+        <v/>
       </c>
     </row>
     <row r="158">
@@ -2611,13 +2611,13 @@
         <v>📥</v>
       </c>
       <c r="B158" t="str">
-        <v>BL-047: תווית "כרגע ניתן לייבא קובץ CSV בלבד" מוצגת ליד אזור ההעלאה ב-ImportContactsScreen; תרגום עברי קיים</v>
+        <v>BL-046: כפתור ייבוא אנשי קשר מוצג בכרטיסיית אנשי קשר לכל המשתמשים; גייט Premium נשמר בנתיב /import</v>
       </c>
       <c r="C158" t="str">
         <v>✅</v>
       </c>
       <c r="D158" t="str">
-        <v>BL-047 אומת — תווית CSV בלבד מוצגת ליד אזור ההעלאה; תרגום עברי קיים</v>
+        <v>BL-046 תוקן — כפתור ייבוא בכרטיסיית אנשי קשר מוצג לכל המשתמשים; גייט Premium נשמר בנתיב</v>
       </c>
     </row>
     <row r="159">
@@ -2625,27 +2625,27 @@
         <v>📥</v>
       </c>
       <c r="B159" t="str">
-        <v>BL-048: כרטיסיית ייבוא ממכשיר (גרדיאנט כחול, סמארטפון) מוצגת בראש ImportContactsScreen; נגישות ויזואלית מלאה</v>
+        <v>BL-047: תווית "כרגע ניתן לייבא קובץ CSV בלבד" מוצגת ליד אזור ההעלאה ב-ImportContactsScreen; תרגום עברי קיים</v>
       </c>
       <c r="C159" t="str">
         <v>✅</v>
       </c>
       <c r="D159" t="str">
-        <v>BL-048 אומת — כרטיסיית ייבוא ממכשיר מוצגת בראש המסך עם גרדיאנט כחול ואייקון סמארטפון</v>
+        <v>BL-047 אומת — תווית CSV בלבד מוצגת ליד אזור ההעלאה; תרגום עברי קיים</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>👤</v>
+        <v>📥</v>
       </c>
       <c r="B160" t="str">
-        <v>Sprint 16 — שכבת משתמש אישית BL-067: UserSetupScreen, dashboard_hello, pendingItems</v>
+        <v>BL-048: כרטיסיית ייבוא ממכשיר (גרדיאנט כחול, סמארטפון) מוצגת בראש ImportContactsScreen; נגישות ויזואלית מלאה</v>
       </c>
       <c r="C160" t="str">
-        <v/>
+        <v>✅</v>
       </c>
       <c r="D160" t="str">
-        <v/>
+        <v>BL-048 אומת — כרטיסיית ייבוא ממכשיר מוצגת בראש המסך עם גרדיאנט כחול ואייקון סמארטפון</v>
       </c>
     </row>
     <row r="161">
@@ -2653,19 +2653,33 @@
         <v>👤</v>
       </c>
       <c r="B161" t="str">
+        <v>Sprint 16 — שכבת משתמש אישית BL-067: UserSetupScreen, dashboard_hello, pendingItems</v>
+      </c>
+      <c r="C161" t="str">
+        <v/>
+      </c>
+      <c r="D161" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="str">
+        <v>👤</v>
+      </c>
+      <c r="B162" t="str">
         <v>BL-067: UserSetupScreen first-launch, nm_user_name persist, dashboard_hello/pending/first_greeting EN+HE, pendingItems clickable, empty states graceful; DoD מלא ✅</v>
       </c>
-      <c r="C161" t="str">
-        <v>✅</v>
-      </c>
-      <c r="D161" t="str">
+      <c r="C162" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D162" t="str">
         <v>BL-067 DoD מלא אומת — UserSetupScreen first-launch, nm_user_name persist, dashboard_hello/pending/first_greeting keys EN+HE, pendingItems clickable, empty states graceful</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D161"/>
+  <autoFilter ref="A1:D162"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D161"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D162"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(sprint23): Group delete cleanup, subtitle fix, group filter chip (BL-086/088/087)
- BL-086: deleteContact now removes contact ID from all groups' contactIds
- BL-088: ContactsScreen subtitle uses contacts_contact/contacts_contacts keys (EN+HE)
- BL-087: Active group filter chip in ContactsScreen — shows group name + emoji from ?group= param, X button clears filter

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NeverMiss_QA_Checklist.xlsx
+++ b/NeverMiss_QA_Checklist.xlsx
@@ -6,7 +6,7 @@
     <sheet name="QA Checklist" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D162</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'QA Checklist'!A1:D184</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D162"/>
+  <dimension ref="A1:D184"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="52.83203125" customWidth="1"/>
@@ -2676,10 +2676,318 @@
         <v>BL-067 DoD מלא אומת — UserSetupScreen first-launch, nm_user_name persist, dashboard_hello/pending/first_greeting keys EN+HE, pendingItems clickable, empty states graceful</v>
       </c>
     </row>
+    <row r="163">
+      <c r="A163" t="str">
+        <v>🔧</v>
+      </c>
+      <c r="B163" t="str">
+        <v>Sprint 17 — BL-075: תיקוני BugHunter</v>
+      </c>
+      <c r="C163" t="str">
+        <v/>
+      </c>
+      <c r="D163" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="str">
+        <v>📱</v>
+      </c>
+      <c r="B164" t="str">
+        <v>Sprint 18 — RTL icons, contact card overflow, BottomNav active indicator</v>
+      </c>
+      <c r="C164" t="str">
+        <v/>
+      </c>
+      <c r="D164" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="str">
+        <v>📱</v>
+      </c>
+      <c r="B165" t="str">
+        <v>BL-081: ImportContactsScreen — 3 ArrowRight הוחלפו ב-lang==="he" ? ArrowLeft : ArrowRight; כפתור מכשיר, הורד תבנית, עמודת מיפוי כולם RTL-נכון</v>
+      </c>
+      <c r="C165" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D165" t="str">
+        <v>BL-081 תוקן — ImportContactsScreen: 3 מופעי ArrowRight הוחלפו ב-lang==='he' ? ArrowLeft : ArrowRight; useLang() נוסף; build+lint ✅</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="str">
+        <v>📱</v>
+      </c>
+      <c r="B166" t="str">
+        <v>BL-075: ContactCard — 3-dot MoreVertical menu; Edit מנווט לטופס; Delete פותח confirm modal; סגירה על-ידי outside click + Escape; aria-label; dropdown RTL-aware</v>
+      </c>
+      <c r="C166" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D166" t="str">
+        <v>BL-075 יושם — ContactCard: 3-dot MoreVertical menu עם Edit+Delete; close on outside click + Escape; delete confirmation modal; aria-label contacts_moreOptions; RTL-correct dropdown position; build+lint ✅</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="str">
+        <v>📱</v>
+      </c>
+      <c r="B167" t="str">
+        <v>BL-049: BottomNav active tab — box-shadow inset 0 2px 0 var(--color-primary) + opacity-20 icon glow; active tab ברור ומובחן; ללא רגרסיה</v>
+      </c>
+      <c r="C167" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D167" t="str">
+        <v>BL-049 שופר — BottomNav active tab: box-shadow inset 0 2px 0 var(--color-primary) נוסף; opacity-20 (מ-15); active indication ברור יותר; build+lint ✅</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="str">
+        <v>🌐</v>
+      </c>
+      <c r="B168" t="str">
+        <v>Sprint 19 — BL-079: Language-Religion drilldown + CSV localization</v>
+      </c>
+      <c r="C168" t="str">
+        <v/>
+      </c>
+      <c r="D168" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="str">
+        <v>🌐</v>
+      </c>
+      <c r="B169" t="str">
+        <v>BL-079: contactConfig.ts single source of truth; normalizeLanguage/normalizeReligion מקבלים raw key / EN label / HE label; CSV template מלוקלי לפי app lang; Religion dropdown ב-ContactForm מסודר לפי שפת הקשר; build+lint ✅</v>
+      </c>
+      <c r="C169" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D169" t="str">
+        <v>BL-079 יושם — contactConfig.ts: LANGUAGE_KEYS/RELIGION_KEYS/LANGUAGE_RELIGION_ORDER/normalizeLanguage/normalizeReligion/getLanguageDisplayValue/getReligionDisplayValue; importService.ts: normalizeLanguage+normalizeReligion במקום cast ישיר; ImportContactsScreen.tsx: CSV headers+example row מלוקלים לפי lang; ContactFormScreen.tsx: Religion dropdown מסודר לפי LANGUAGE_RELIGION_ORDER; build+lint ✅; normalization tests ✅</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="str">
+        <v>📅</v>
+      </c>
+      <c r="B170" t="str">
+        <v>Sprint 20 — BL-076: Hebrew Birthday import/export round-trip</v>
+      </c>
+      <c r="C170" t="str">
+        <v/>
+      </c>
+      <c r="D170" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="str">
+        <v>📅</v>
+      </c>
+      <c r="B171" t="str">
+        <v>BL-076: Hebrew Birthday column בתבנית CSV (EN+HE); DETECTABLE_FIELDS: hebrewBirthday לפני birthday; processImport כותב hebrewBirthday; round-trip export↔import תקין; build+lint ✅</v>
+      </c>
+      <c r="C171" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D171" t="str">
+        <v>BL-076 יושם — importService.ts: hebrewBirthday ב-DETECTABLE_FIELDS (לפני birthday) + processImport; ImportContactsScreen.tsx: עמודת Hebrew Birthday (DD-MM) בתבנית EN+HE; round-trip export↔import תקין; build+lint ✅</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="str">
+        <v>👥</v>
+      </c>
+      <c r="B172" t="str">
+        <v>Sprint 21 — BL-084/082/068/069: Import fix, Score tooltip, Group members, Assign group</v>
+      </c>
+      <c r="C172" t="str">
+        <v/>
+      </c>
+      <c r="D172" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="str">
+        <v>👥</v>
+      </c>
+      <c r="B173" t="str">
+        <v>BL-084: normalizeBirthday() ב-importService.ts; isNaN guard ב-ContactDetailScreen.tsx; קשר מיובא עם תאריך לא-ISO נפתח ללא קריסה; build+lint ✅</v>
+      </c>
+      <c r="C173" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D173" t="str">
+        <v>BL-084 תוקן — normalizeBirthday() ב-importService.ts; isNaN guard ב-ContactDetailScreen.tsx; מונע קריסה על תאריכים בפורמט שגוי; build+lint ✅</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="str">
+        <v>👥</v>
+      </c>
+      <c r="B174" t="str">
+        <v>BL-082: תג ציון ב-ContactCard הפך ל-button; לחיצה מציגה tooltip עם הסבר ציון; click-outside/Escape סוגרים; EN+HE; build+lint ✅</v>
+      </c>
+      <c r="C174" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D174" t="str">
+        <v>BL-082 יושם — תג הציון ב-ContactCard הפך ל-button; tooltip עם score_tipTitle/score_tipBody בלחיצה; EN+HE; click-outside סוגר; build+lint ✅</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="str">
+        <v>👥</v>
+      </c>
+      <c r="B175" t="str">
+        <v>BL-068: contact picker ב-GroupsScreen modal (Premium); selectedContactIds נשמרים ב-handleSave; חיפוש אנשי קשר; EN+HE; build+lint ✅</v>
+      </c>
+      <c r="C175" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D175" t="str">
+        <v>BL-068 יושם — contact picker ב-GroupsScreen modal; selectedContactIds state; openForm מאתחל מ-group.contactIds; handleSave שומר; EN+HE; build+lint ✅</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="str">
+        <v>👥</v>
+      </c>
+      <c r="B176" t="str">
+        <v>BL-069: group selector ב-ContactFormScreen לאנשי קשר חדשים; לאחר addContact מעדכן group.contactIds; EN+HE; build+lint ✅</v>
+      </c>
+      <c r="C176" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D176" t="str">
+        <v>BL-069 יושם — group selector ב-ContactFormScreen (חדש בלבד); לאחר addContact מעדכן group.contactIds; EN+HE; build+lint ✅</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="str">
+        <v>📦</v>
+      </c>
+      <c r="B177" t="str">
+        <v>Sprint 22 — BL-092/090/091: Import celebrationType + hebrewBirthday + export warning</v>
+      </c>
+      <c r="C177" t="str">
+        <v/>
+      </c>
+      <c r="D177" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="str">
+        <v>📦</v>
+      </c>
+      <c r="B178" t="str">
+        <v>BL-092: celebrationType ב-DETECTABLE_FIELDS; normalizeCelebrationType(); processImport כותב celebrationType; round-trip export-import תקין; build+lint ✅</v>
+      </c>
+      <c r="C178" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D178" t="str">
+        <v>BL-092 יושם — celebrationType ב-DETECTABLE_FIELDS; normalizeCelebrationType() ממפה ערכים; processImport כותב celebrationType; round-trip export-import תקין; build+lint ✅</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="str">
+        <v>📦</v>
+      </c>
+      <c r="B179" t="str">
+        <v>BL-090: normalizeHebrewBirthday() מאמת DD-MM בייבוא; regex guard ב-ContactDetailScreen; ערכים לא תקינים לא מוצגים; build+lint ✅</v>
+      </c>
+      <c r="C179" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D179" t="str">
+        <v>BL-090 יושם — normalizeHebrewBirthday() מאמת פורמט DD-MM בייבוא; regex guard ב-ContactDetailScreen מונע הצגת ערך לא תקין; build+lint ✅</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="str">
+        <v>📦</v>
+      </c>
+      <c r="B180" t="str">
+        <v>BL-091: settings_exportGroupWarning EN+HE; אזהרה מתחת לכפתור ייצוא CSV ב-SettingsScreen; build+lint ✅</v>
+      </c>
+      <c r="C180" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D180" t="str">
+        <v>BL-091 יושם — settings_exportGroupWarning EN+HE; טקסט אזהרה מתחת לכפתור ייצוא CSV ב-SettingsScreen; build+lint ✅</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="str">
+        <v>🧹</v>
+      </c>
+      <c r="B181" t="str">
+        <v>Sprint 23 — BL-086/088/087: Group delete cleanup, subtitle fix, group filter chip</v>
+      </c>
+      <c r="C181" t="str">
+        <v/>
+      </c>
+      <c r="D181" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="str">
+        <v>🧹</v>
+      </c>
+      <c r="B182" t="str">
+        <v>BL-086: deleteContact מנקה contactIds בקבוצות; שלמות נתונים נשמרת; build+lint ✅</v>
+      </c>
+      <c r="C182" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D182" t="str">
+        <v>BL-086 תוקן — deleteContact ב-AppContext.tsx מנקה כעת contactIds בכל קבוצה שמכילה את המזהה שנמחק; שלמות נתונים נשמרת; build+lint ✅</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="str">
+        <v>🧹</v>
+      </c>
+      <c r="B183" t="str">
+        <v>BL-088: כותרת משנה ב-ContactsScreen — contacts_contact/contacts_contacts EN+HE; תיקון מפתחות i18n; build+lint ✅</v>
+      </c>
+      <c r="C183" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D183" t="str">
+        <v>BL-088 תוקן — כותרת המשנה ב-ContactsScreen מציגה 'X אנשי קשר' במקום 'X קבוצות'; מפתחות contacts_contact/contacts_contacts EN+HE; build+lint ✅</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="str">
+        <v>🧹</v>
+      </c>
+      <c r="B184" t="str">
+        <v>BL-087: chip סינון קבוצה ב-ContactsScreen; ?group=X מסנן + מציג chip; כפתור ניקוי; build+lint ✅</v>
+      </c>
+      <c r="C184" t="str">
+        <v>✅</v>
+      </c>
+      <c r="D184" t="str">
+        <v>BL-087 יושם — chip סינון קבוצה ב-ContactsScreen: מוצג כש-?group=X; שם הקבוצה + אמוג'י + כפתור ניקוי; הרשימה מסוננת; build+lint ✅</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D162"/>
+  <autoFilter ref="A1:D184"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D162"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D184"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>